<commit_message>
Refactor and update economic analysis plotting scripts
Major refactor of R plotting code for economic and ecological multifunctionality analyses. Adds new custom theme, updates plot generation for SGM, SOC, leaching, and total costs, and improves code structure and clarity. Removes obsolete scripts and data files, and adds new output figures for realized plant diversity effects. Minor updates to R project user settings and source tracking.
</commit_message>
<xml_diff>
--- a/Data Analysis/1_Data/Aggregates/Results_Spring2024_WSA_all.xlsx
+++ b/Data Analysis/1_Data/Aggregates/Results_Spring2024_WSA_all.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mm68tulo\Desktop\Jena Chapter\Data Analysis\1_Data\Aggregates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D074A178-7A72-4CC0-A7CD-872E10A7E00E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99E28134-19A1-4012-9787-1FB29FED4114}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1230" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1230" uniqueCount="110">
   <si>
     <t>Number</t>
   </si>
@@ -386,6 +386,9 @@
   </si>
   <si>
     <t>agg_overall</t>
+  </si>
+  <si>
+    <t>WSA</t>
   </si>
 </sst>
 </file>
@@ -839,7 +842,7 @@
         <v>9</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>10</v>
+        <v>109</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>11</v>

</xml_diff>